<commit_message>
updated the tests to reflect changes to giulia's test, ran new bvar specifications for alignment with qr and produced new test results
</commit_message>
<xml_diff>
--- a/IaR_GaR_April_2026/Outputs/forecast_evaluation/comparison_fcst_eval_growth.xlsx
+++ b/IaR_GaR_April_2026/Outputs/forecast_evaluation/comparison_fcst_eval_growth.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="193">
   <si>
     <t>horizon</t>
   </si>
@@ -408,6 +408,204 @@
   </si>
   <si>
     <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_1</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_2</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_3</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_1</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_2</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_3</t>
   </si>
 </sst>
 </file>
@@ -465,16 +663,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>74</v>
+        <v>130</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -491,7 +689,7 @@
         <v>0.19042743907996229</v>
       </c>
       <c r="D2" s="0">
-        <v>0.19528968220564347</v>
+        <v>0.19872237201324139</v>
       </c>
       <c r="E2" s="0">
         <v>0.15591199773247905</v>
@@ -508,7 +706,7 @@
         <v>0.1504135714879189</v>
       </c>
       <c r="D3" s="0">
-        <v>0.18277082151778923</v>
+        <v>0.10712541201019532</v>
       </c>
       <c r="E3" s="0">
         <v>0.27295529855764578</v>
@@ -525,7 +723,7 @@
         <v>0.20169170657447</v>
       </c>
       <c r="D4" s="0">
-        <v>0.24742932092734116</v>
+        <v>0.13555703999015145</v>
       </c>
       <c r="E4" s="0">
         <v>0.34750008907715058</v>
@@ -542,7 +740,7 @@
         <v>0.22397972850475989</v>
       </c>
       <c r="D5" s="0">
-        <v>0.26778041316153073</v>
+        <v>0.10144397192505794</v>
       </c>
       <c r="E5" s="0">
         <v>0.35925314693549149</v>
@@ -559,7 +757,7 @@
         <v>0.28594408866230941</v>
       </c>
       <c r="D6" s="0">
-        <v>0.28900685160468542</v>
+        <v>0.1182617078629899</v>
       </c>
       <c r="E6" s="0">
         <v>0.41659379434822996</v>
@@ -576,7 +774,7 @@
         <v>0.35199484598127867</v>
       </c>
       <c r="D7" s="0">
-        <v>0.36659949568749228</v>
+        <v>0.1708827942298406</v>
       </c>
       <c r="E7" s="0">
         <v>0.56496203003384826</v>
@@ -593,7 +791,7 @@
         <v>0.32187935206638957</v>
       </c>
       <c r="D8" s="0">
-        <v>0.40732985329200311</v>
+        <v>0.20344751165240638</v>
       </c>
       <c r="E8" s="0">
         <v>0.57394609820231468</v>
@@ -610,7 +808,7 @@
         <v>0.36187354213386153</v>
       </c>
       <c r="D9" s="0">
-        <v>0.39279924721648096</v>
+        <v>0.22127373203268186</v>
       </c>
       <c r="E9" s="0">
         <v>0.55262569690000662</v>
@@ -627,7 +825,7 @@
         <v>0.2978827399962517</v>
       </c>
       <c r="D10" s="0">
-        <v>0.33929752641304667</v>
+        <v>0.18640164647697341</v>
       </c>
       <c r="E10" s="0">
         <v>0.53854002133050705</v>
@@ -644,7 +842,7 @@
         <v>0.26042813027814826</v>
       </c>
       <c r="D11" s="0">
-        <v>0.27238711624176359</v>
+        <v>0.23963330288479226</v>
       </c>
       <c r="E11" s="0">
         <v>0.43232379483671357</v>
@@ -661,7 +859,7 @@
         <v>0.25603354211073448</v>
       </c>
       <c r="D12" s="0">
-        <v>0.22139964042730431</v>
+        <v>0.26642939342032113</v>
       </c>
       <c r="E12" s="0">
         <v>0.39229897896382715</v>
@@ -678,7 +876,7 @@
         <v>0.19197662244303593</v>
       </c>
       <c r="D13" s="0">
-        <v>0.18738247268664709</v>
+        <v>0.25363320059758288</v>
       </c>
       <c r="E13" s="0">
         <v>0.37313397830086764</v>
@@ -695,7 +893,7 @@
         <v>0.21241242933645166</v>
       </c>
       <c r="D14" s="0">
-        <v>0.23146430357573189</v>
+        <v>0.25459506983989766</v>
       </c>
       <c r="E14" s="0">
         <v>0.48590913364244048</v>
@@ -713,22 +911,22 @@
     <col min="1" max="1" width="7.85546875" customWidth="true"/>
     <col min="2" max="2" width="13.7109375" customWidth="true"/>
     <col min="3" max="3" width="13.7109375" customWidth="true"/>
-    <col min="4" max="4" width="13.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="14.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>107</v>
+        <v>163</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>108</v>
+        <v>164</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>110</v>
+        <v>166</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -745,7 +943,7 @@
         <v>0.040861441346580096</v>
       </c>
       <c r="D2" s="0">
-        <v>0.21311516804565189</v>
+        <v>0.18079793700867575</v>
       </c>
       <c r="E2" s="0">
         <v>0.68831213837965133</v>
@@ -762,7 +960,7 @@
         <v>0.3499015278032358</v>
       </c>
       <c r="D3" s="0">
-        <v>0.10137968663420716</v>
+        <v>0.30978646174982716</v>
       </c>
       <c r="E3" s="0">
         <v>0.22544002930494411</v>
@@ -779,7 +977,7 @@
         <v>0.12812978817280407</v>
       </c>
       <c r="D4" s="0">
-        <v>0.066553138230247111</v>
+        <v>0.27597770764792551</v>
       </c>
       <c r="E4" s="0">
         <v>0.28818793523641051</v>
@@ -796,7 +994,7 @@
         <v>0.090306168490604466</v>
       </c>
       <c r="D5" s="0">
-        <v>0.144187928461464</v>
+        <v>0.30158974566396723</v>
       </c>
       <c r="E5" s="0">
         <v>0.062855343373911632</v>
@@ -813,7 +1011,7 @@
         <v>0.1567451803233213</v>
       </c>
       <c r="D6" s="0">
-        <v>0.173837641152077</v>
+        <v>0.31364761021731735</v>
       </c>
       <c r="E6" s="0">
         <v>0.07068156475293097</v>
@@ -830,7 +1028,7 @@
         <v>0.15642457466498805</v>
       </c>
       <c r="D7" s="0">
-        <v>0.24757662359272214</v>
+        <v>0.32050032912016291</v>
       </c>
       <c r="E7" s="0">
         <v>0.0096007437802668738</v>
@@ -847,7 +1045,7 @@
         <v>0.10946686573774889</v>
       </c>
       <c r="D8" s="0">
-        <v>0.36640191956100954</v>
+        <v>0.46310665488967573</v>
       </c>
       <c r="E8" s="0">
         <v>0.0041022074669080366</v>
@@ -864,7 +1062,7 @@
         <v>0.17082870123571225</v>
       </c>
       <c r="D9" s="0">
-        <v>0.42036874274727265</v>
+        <v>0.45156480242670283</v>
       </c>
       <c r="E9" s="0">
         <v>0.0039342356736554729</v>
@@ -881,7 +1079,7 @@
         <v>0.29624524980235356</v>
       </c>
       <c r="D10" s="0">
-        <v>0.5103199303494883</v>
+        <v>0.50531215314252376</v>
       </c>
       <c r="E10" s="0">
         <v>0.013587201663587956</v>
@@ -898,7 +1096,7 @@
         <v>0.5260153193748236</v>
       </c>
       <c r="D11" s="0">
-        <v>0.40795410531987608</v>
+        <v>0.50242160401569147</v>
       </c>
       <c r="E11" s="0">
         <v>0.036188908936314323</v>
@@ -915,7 +1113,7 @@
         <v>0.45313436626608816</v>
       </c>
       <c r="D12" s="0">
-        <v>0.24276946426442847</v>
+        <v>0.17612139611675115</v>
       </c>
       <c r="E12" s="0">
         <v>0.039858372347144955</v>
@@ -932,7 +1130,7 @@
         <v>0.53008543088784188</v>
       </c>
       <c r="D13" s="0">
-        <v>0.17437083556969757</v>
+        <v>0.39089006678185068</v>
       </c>
       <c r="E13" s="0">
         <v>0.015058227979301897</v>
@@ -949,7 +1147,7 @@
         <v>0.44578043386097388</v>
       </c>
       <c r="D14" s="0">
-        <v>0.23396031947262286</v>
+        <v>0.38007983534902268</v>
       </c>
       <c r="E14" s="0">
         <v>0.023249768241102586</v>
@@ -973,16 +1171,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>111</v>
+        <v>167</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -999,7 +1197,7 @@
         <v>15.82192835928117</v>
       </c>
       <c r="D2" s="0">
-        <v>4.0032542743264541</v>
+        <v>4.781957802566505</v>
       </c>
       <c r="E2" s="0">
         <v>5.6345185290204354</v>
@@ -1016,7 +1214,7 @@
         <v>10.46746225873884</v>
       </c>
       <c r="D3" s="0">
-        <v>6.9213533452461649</v>
+        <v>7.8289441251201408</v>
       </c>
       <c r="E3" s="0">
         <v>5.8108121299644804</v>
@@ -1033,7 +1231,7 @@
         <v>9.5495873928723984</v>
       </c>
       <c r="D4" s="0">
-        <v>9.4342579176117898</v>
+        <v>5.052362894059697</v>
       </c>
       <c r="E4" s="0">
         <v>4.3791804766078233</v>
@@ -1050,7 +1248,7 @@
         <v>9.3414550872306528</v>
       </c>
       <c r="D5" s="0">
-        <v>6.7972159573074356</v>
+        <v>7.199010558360297</v>
       </c>
       <c r="E5" s="0">
         <v>9.986218998589381</v>
@@ -1067,7 +1265,7 @@
         <v>4.7194310605114298</v>
       </c>
       <c r="D6" s="0">
-        <v>9.0585344351617341</v>
+        <v>4.8047262952404886</v>
       </c>
       <c r="E6" s="0">
         <v>8.195951297559132</v>
@@ -1084,7 +1282,7 @@
         <v>6.8412602823854787</v>
       </c>
       <c r="D7" s="0">
-        <v>7.0538962357389439</v>
+        <v>5.8999011544917783</v>
       </c>
       <c r="E7" s="0">
         <v>16.830030008973527</v>
@@ -1101,7 +1299,7 @@
         <v>11.349975271077838</v>
       </c>
       <c r="D8" s="0">
-        <v>10.084045641856228</v>
+        <v>5.0913391681054181</v>
       </c>
       <c r="E8" s="0">
         <v>11.574472374073373</v>
@@ -1118,7 +1316,7 @@
         <v>7.1469607856794353</v>
       </c>
       <c r="D9" s="0">
-        <v>8.6037762696578586</v>
+        <v>7.8270578390721735</v>
       </c>
       <c r="E9" s="0">
         <v>13.248164803714937</v>
@@ -1135,7 +1333,7 @@
         <v>6.3892371751934274</v>
       </c>
       <c r="D10" s="0">
-        <v>6.5883295803771622</v>
+        <v>4.2673077236579182</v>
       </c>
       <c r="E10" s="0">
         <v>16.77007149986245</v>
@@ -1152,7 +1350,7 @@
         <v>5.4737174269237494</v>
       </c>
       <c r="D11" s="0">
-        <v>4.6954331884756968</v>
+        <v>4.5339288110797886</v>
       </c>
       <c r="E11" s="0">
         <v>9.5235415644985757</v>
@@ -1169,7 +1367,7 @@
         <v>2.7599610028432462</v>
       </c>
       <c r="D12" s="0">
-        <v>9.659520506900213</v>
+        <v>4.8893005182491596</v>
       </c>
       <c r="E12" s="0">
         <v>8.6934914039679629</v>
@@ -1186,7 +1384,7 @@
         <v>3.2404909078550901</v>
       </c>
       <c r="D13" s="0">
-        <v>8.8031042631781737</v>
+        <v>5.8348317265378586</v>
       </c>
       <c r="E13" s="0">
         <v>10.263900367645462</v>
@@ -1203,7 +1401,7 @@
         <v>4.2101798133626591</v>
       </c>
       <c r="D14" s="0">
-        <v>8.6192913236775937</v>
+        <v>4.4538969084145617</v>
       </c>
       <c r="E14" s="0">
         <v>13.403385961619186</v>
@@ -1221,22 +1419,22 @@
     <col min="1" max="1" width="7.85546875" customWidth="true"/>
     <col min="2" max="2" width="13.7109375" customWidth="true"/>
     <col min="3" max="3" width="14.7109375" customWidth="true"/>
-    <col min="4" max="4" width="13.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="14.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>115</v>
+        <v>171</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>116</v>
+        <v>172</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>117</v>
+        <v>173</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>118</v>
+        <v>174</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -1253,7 +1451,7 @@
         <v>0.0073713006231521661</v>
       </c>
       <c r="D2" s="0">
-        <v>0.54894750960427818</v>
+        <v>0.44306577034312533</v>
       </c>
       <c r="E2" s="0">
         <v>0.34342076316334647</v>
@@ -1270,7 +1468,7 @@
         <v>0.063022960106911774</v>
       </c>
       <c r="D3" s="0">
-        <v>0.22655538104628326</v>
+        <v>0.16591823478856416</v>
       </c>
       <c r="E3" s="0">
         <v>0.32506518980700383</v>
@@ -1287,7 +1485,7 @@
         <v>0.089050991537168112</v>
       </c>
       <c r="D4" s="0">
-        <v>0.092947178029276656</v>
+        <v>0.40952325840573534</v>
       </c>
       <c r="E4" s="0">
         <v>0.49620953346307051</v>
@@ -1304,7 +1502,7 @@
         <v>0.096195566385820719</v>
       </c>
       <c r="D5" s="0">
-        <v>0.23616371508040046</v>
+        <v>0.2062553869855861</v>
       </c>
       <c r="E5" s="0">
         <v>0.075626667730786079</v>
@@ -1321,7 +1519,7 @@
         <v>0.45107125756402067</v>
       </c>
       <c r="D6" s="0">
-        <v>0.10675207022273914</v>
+        <v>0.44017362950536276</v>
       </c>
       <c r="E6" s="0">
         <v>0.14576189389809269</v>
@@ -1338,7 +1536,7 @@
         <v>0.23271620589900577</v>
       </c>
       <c r="D7" s="0">
-        <v>0.21666273924739599</v>
+        <v>0.31608116880835879</v>
       </c>
       <c r="E7" s="0">
         <v>0.0048336893567137995</v>
@@ -1355,7 +1553,7 @@
         <v>0.044865966985496941</v>
       </c>
       <c r="D8" s="0">
-        <v>0.072888575834855418</v>
+        <v>0.40483512511510722</v>
       </c>
       <c r="E8" s="0">
         <v>0.041107364063473373</v>
@@ -1372,7 +1570,7 @@
         <v>0.20993808632549316</v>
       </c>
       <c r="D9" s="0">
-        <v>0.12595070325310753</v>
+        <v>0.16602789368219673</v>
       </c>
       <c r="E9" s="0">
         <v>0.021160928124125289</v>
@@ -1389,7 +1587,7 @@
         <v>0.27016473843792077</v>
       </c>
       <c r="D10" s="0">
-        <v>0.25310024952240395</v>
+        <v>0.51160647182243757</v>
       </c>
       <c r="E10" s="0">
         <v>0.0049571508387528107</v>
@@ -1406,7 +1604,7 @@
         <v>0.36083646851955975</v>
       </c>
       <c r="D11" s="0">
-        <v>0.45416818752724286</v>
+        <v>0.47535675437844516</v>
       </c>
       <c r="E11" s="0">
         <v>0.089917509329231149</v>
@@ -1423,7 +1621,7 @@
         <v>0.73693349696535093</v>
       </c>
       <c r="D12" s="0">
-        <v>0.085477826738126317</v>
+        <v>0.42953908225346549</v>
       </c>
       <c r="E12" s="0">
         <v>0.12193222683556937</v>
@@ -1440,7 +1638,7 @@
         <v>0.66296408016873964</v>
       </c>
       <c r="D13" s="0">
-        <v>0.11718012076884676</v>
+        <v>0.32262375451351932</v>
       </c>
       <c r="E13" s="0">
         <v>0.068093884634720658</v>
@@ -1457,7 +1655,7 @@
         <v>0.51956912338116601</v>
       </c>
       <c r="D14" s="0">
-        <v>0.12524731932837119</v>
+        <v>0.48607546972555882</v>
       </c>
       <c r="E14" s="0">
         <v>0.01987805158127931</v>
@@ -1481,16 +1679,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>119</v>
+        <v>175</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>122</v>
+        <v>178</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -1507,7 +1705,7 @@
         <v>0.1679837152354782</v>
       </c>
       <c r="D2" s="0">
-        <v>0.27913923107813238</v>
+        <v>0.2809489921158797</v>
       </c>
       <c r="E2" s="0">
         <v>0.50647631546024863</v>
@@ -1524,7 +1722,7 @@
         <v>0.62650335780909627</v>
       </c>
       <c r="D3" s="0">
-        <v>0.62866322796012997</v>
+        <v>0.62167181402044225</v>
       </c>
       <c r="E3" s="0">
         <v>0.57095405101496277</v>
@@ -1541,7 +1739,7 @@
         <v>1.0035089010902936</v>
       </c>
       <c r="D4" s="0">
-        <v>0.97927444156147359</v>
+        <v>0.96072627215794892</v>
       </c>
       <c r="E4" s="0">
         <v>0.98155429835630481</v>
@@ -1558,7 +1756,7 @@
         <v>1.1895925603145583</v>
       </c>
       <c r="D5" s="0">
-        <v>1.2755619523573429</v>
+        <v>1.2458289507693914</v>
       </c>
       <c r="E5" s="0">
         <v>1.2713224172669342</v>
@@ -1575,7 +1773,7 @@
         <v>1.252434345172609</v>
       </c>
       <c r="D6" s="0">
-        <v>1.4832971168818632</v>
+        <v>1.4621751463874488</v>
       </c>
       <c r="E6" s="0">
         <v>1.302399546160403</v>
@@ -1592,7 +1790,7 @@
         <v>1.2407009705663441</v>
       </c>
       <c r="D7" s="0">
-        <v>1.5622791621636074</v>
+        <v>1.5555692831286236</v>
       </c>
       <c r="E7" s="0">
         <v>1.3713177621214958</v>
@@ -1609,7 +1807,7 @@
         <v>1.2107803475030869</v>
       </c>
       <c r="D8" s="0">
-        <v>1.5514282198417895</v>
+        <v>1.5703368015237504</v>
       </c>
       <c r="E8" s="0">
         <v>1.4450424410809661</v>
@@ -1626,7 +1824,7 @@
         <v>1.1180936887022808</v>
       </c>
       <c r="D9" s="0">
-        <v>1.4521745301367883</v>
+        <v>1.4819285520547654</v>
       </c>
       <c r="E9" s="0">
         <v>1.4551603297551585</v>
@@ -1643,7 +1841,7 @@
         <v>0.98562145936125656</v>
       </c>
       <c r="D10" s="0">
-        <v>1.3259303350079588</v>
+        <v>1.3502779223169923</v>
       </c>
       <c r="E10" s="0">
         <v>1.4439038888194222</v>
@@ -1660,7 +1858,7 @@
         <v>0.84695678226945526</v>
       </c>
       <c r="D11" s="0">
-        <v>1.1965065371744072</v>
+        <v>1.2450496235625037</v>
       </c>
       <c r="E11" s="0">
         <v>1.4255902921749017</v>
@@ -1677,7 +1875,7 @@
         <v>0.8180318850141084</v>
       </c>
       <c r="D12" s="0">
-        <v>1.0951205228844281</v>
+        <v>1.1846320830882715</v>
       </c>
       <c r="E12" s="0">
         <v>1.4562601751235482</v>
@@ -1694,7 +1892,7 @@
         <v>0.83585118851254181</v>
       </c>
       <c r="D13" s="0">
-        <v>1.044260573842432</v>
+        <v>1.1773074868025273</v>
       </c>
       <c r="E13" s="0">
         <v>1.5105726857697219</v>
@@ -1711,7 +1909,7 @@
         <v>0.82138479793964558</v>
       </c>
       <c r="D14" s="0">
-        <v>1.0870645493448594</v>
+        <v>1.2693980482630896</v>
       </c>
       <c r="E14" s="0">
         <v>1.5417742712901181</v>
@@ -1735,16 +1933,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>124</v>
+        <v>180</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>125</v>
+        <v>181</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -1761,7 +1959,7 @@
         <v>0.054472937433764211</v>
       </c>
       <c r="D2" s="0">
-        <v>0.095885094167423607</v>
+        <v>0.096757618588159608</v>
       </c>
       <c r="E2" s="0">
         <v>0.13478902349114597</v>
@@ -1778,7 +1976,7 @@
         <v>0.21669427808708719</v>
       </c>
       <c r="D3" s="0">
-        <v>0.20822880770250804</v>
+        <v>0.2068204529785985</v>
       </c>
       <c r="E3" s="0">
         <v>0.15939997405061687</v>
@@ -1795,7 +1993,7 @@
         <v>0.34523645393770763</v>
       </c>
       <c r="D4" s="0">
-        <v>0.31686311628029862</v>
+        <v>0.31266497930054438</v>
       </c>
       <c r="E4" s="0">
         <v>0.35159728555157344</v>
@@ -1812,7 +2010,7 @@
         <v>0.41918952396377063</v>
       </c>
       <c r="D5" s="0">
-        <v>0.40533616779110626</v>
+        <v>0.40576888828641622</v>
       </c>
       <c r="E5" s="0">
         <v>0.41301094073859773</v>
@@ -1829,7 +2027,7 @@
         <v>0.46240295575508972</v>
       </c>
       <c r="D6" s="0">
-        <v>0.46402501146273695</v>
+        <v>0.48328407036722948</v>
       </c>
       <c r="E6" s="0">
         <v>0.41613697888057966</v>
@@ -1846,7 +2044,7 @@
         <v>0.43811680843408496</v>
       </c>
       <c r="D7" s="0">
-        <v>0.47371289369094244</v>
+        <v>0.51964497287978684</v>
       </c>
       <c r="E7" s="0">
         <v>0.43981563109013577</v>
@@ -1863,7 +2061,7 @@
         <v>0.42624211076970031</v>
       </c>
       <c r="D8" s="0">
-        <v>0.45693705910257443</v>
+        <v>0.52664568312986693</v>
       </c>
       <c r="E8" s="0">
         <v>0.45997198127620509</v>
@@ -1880,7 +2078,7 @@
         <v>0.38553769702723906</v>
       </c>
       <c r="D9" s="0">
-        <v>0.41117536484811429</v>
+        <v>0.49472740887684474</v>
       </c>
       <c r="E9" s="0">
         <v>0.4461582129817111</v>
@@ -1897,7 +2095,7 @@
         <v>0.34500558270740328</v>
       </c>
       <c r="D10" s="0">
-        <v>0.36242505499151384</v>
+        <v>0.44504072880290957</v>
       </c>
       <c r="E10" s="0">
         <v>0.43009545178412523</v>
@@ -1914,7 +2112,7 @@
         <v>0.29835717767124248</v>
       </c>
       <c r="D11" s="0">
-        <v>0.32637204803066061</v>
+        <v>0.4133142033288022</v>
       </c>
       <c r="E11" s="0">
         <v>0.43572697137845473</v>
@@ -1931,7 +2129,7 @@
         <v>0.29409205520579113</v>
       </c>
       <c r="D12" s="0">
-        <v>0.30906681684373272</v>
+        <v>0.4046415413462488</v>
       </c>
       <c r="E12" s="0">
         <v>0.43804653191325599</v>
@@ -1948,7 +2146,7 @@
         <v>0.29354924491872697</v>
       </c>
       <c r="D13" s="0">
-        <v>0.30480811925622969</v>
+        <v>0.40914092952429637</v>
       </c>
       <c r="E13" s="0">
         <v>0.46073833193900054</v>
@@ -1965,7 +2163,7 @@
         <v>0.30135306689724511</v>
       </c>
       <c r="D14" s="0">
-        <v>0.32832923230015632</v>
+        <v>0.43839646255327341</v>
       </c>
       <c r="E14" s="0">
         <v>0.49692783668915069</v>
@@ -1991,79 +2189,79 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>61</v>
+        <v>183</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>65</v>
+        <v>187</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>66</v>
+        <v>188</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>67</v>
+        <v>189</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>68</v>
+        <v>190</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>69</v>
+        <v>191</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>70</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>62</v>
+        <v>184</v>
       </c>
       <c r="B2" s="0">
-        <v>1</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="C2" s="0">
-        <v>1</v>
+        <v>0.97399999999999998</v>
       </c>
       <c r="D2" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="0">
         <v>0</v>
       </c>
       <c r="F2" s="0">
-        <v>0.99399999999999999</v>
+        <v>0.1208</v>
       </c>
       <c r="G2" s="0">
-        <v>0.96599999999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>63</v>
+        <v>185</v>
       </c>
       <c r="B3" s="0">
         <v>0</v>
       </c>
       <c r="C3" s="0">
-        <v>0</v>
+        <v>0.0033999999999999998</v>
       </c>
       <c r="D3" s="0">
-        <v>0.033000000000000002</v>
+        <v>0.0014</v>
       </c>
       <c r="E3" s="0">
         <v>0</v>
       </c>
       <c r="F3" s="0">
-        <v>0.64600000000000002</v>
+        <v>0.1232</v>
       </c>
       <c r="G3" s="0">
-        <v>0.097000000000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>64</v>
+        <v>186</v>
       </c>
       <c r="B4" s="0">
-        <v>1</v>
+        <v>0.99360000000000004</v>
       </c>
       <c r="C4" s="0">
         <v>0</v>
@@ -2072,13 +2270,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="0">
-        <v>0.29199999999999998</v>
+        <v>0.0028</v>
       </c>
       <c r="F4" s="0">
         <v>0</v>
       </c>
       <c r="G4" s="0">
-        <v>0</v>
+        <v>0.073599999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2093,22 +2291,22 @@
     <col min="1" max="1" width="7.85546875" customWidth="true"/>
     <col min="2" max="2" width="15.7109375" customWidth="true"/>
     <col min="3" max="3" width="15.7109375" customWidth="true"/>
-    <col min="4" max="4" width="15.7109375" customWidth="true"/>
+    <col min="4" max="4" width="14.7109375" customWidth="true"/>
     <col min="5" max="5" width="15.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>75</v>
+        <v>131</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>78</v>
+        <v>134</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -2125,7 +2323,7 @@
         <v>0.034444556112206502</v>
       </c>
       <c r="D2" s="0">
-        <v>0.025836374268534339</v>
+        <v>0.022143585642230523</v>
       </c>
       <c r="E2" s="0">
         <v>0.13136388183342543</v>
@@ -2142,7 +2340,7 @@
         <v>0.15860297193823761</v>
       </c>
       <c r="D3" s="0">
-        <v>0.047436224533434102</v>
+        <v>0.54143351646348525</v>
       </c>
       <c r="E3" s="0">
         <v>0.00047526262145239281</v>
@@ -2159,7 +2357,7 @@
         <v>0.02281304071027972</v>
       </c>
       <c r="D4" s="0">
-        <v>0.0023829533643045277</v>
+        <v>0.26448283961355312</v>
       </c>
       <c r="E4" s="0">
         <v>2.6738093588918562e-06</v>
@@ -2176,7 +2374,7 @@
         <v>0.008899451746967978</v>
       </c>
       <c r="D5" s="0">
-        <v>0.00087028761071691744</v>
+        <v>0.63517887020697672</v>
       </c>
       <c r="E5" s="0">
         <v>1.0545816544463347e-06</v>
@@ -2193,7 +2391,7 @@
         <v>0.00034705230453133731</v>
       </c>
       <c r="D6" s="0">
-        <v>0.00028800680355986209</v>
+        <v>0.44940386528256104</v>
       </c>
       <c r="E6" s="0">
         <v>7.229193712909694e-09</v>
@@ -2210,7 +2408,7 @@
         <v>5.1501154952018141e-06</v>
       </c>
       <c r="D7" s="0">
-        <v>1.7313704545100471e-06</v>
+        <v>0.096318939092702671</v>
       </c>
       <c r="E7" s="0">
         <v>5.9591835039673681e-16</v>
@@ -2227,7 +2425,7 @@
         <v>5.2337761111001762e-05</v>
       </c>
       <c r="D8" s="0">
-        <v>9.1825360658553663e-08</v>
+        <v>0.029541082747840026</v>
       </c>
       <c r="E8" s="0">
         <v>1.8944119367510097e-16</v>
@@ -2244,7 +2442,7 @@
         <v>4.2176566559314384e-06</v>
       </c>
       <c r="D9" s="0">
-        <v>4.1066033057021658e-07</v>
+        <v>0.015095058111258908</v>
       </c>
       <c r="E9" s="0">
         <v>2.7913798375274149e-15</v>
@@ -2261,7 +2459,7 @@
         <v>0.00034149174991104697</v>
       </c>
       <c r="D10" s="0">
-        <v>2.5877185318229478e-05</v>
+        <v>0.066944843316253541</v>
       </c>
       <c r="E10" s="0">
         <v>1.561155258508762e-14</v>
@@ -2278,7 +2476,7 @@
         <v>0.0034767522055977268</v>
       </c>
       <c r="D11" s="0">
-        <v>0.0019137543165940944</v>
+        <v>0.0092112557223408657</v>
       </c>
       <c r="E11" s="0">
         <v>2.3688754290922974e-09</v>
@@ -2295,7 +2493,7 @@
         <v>0.0056164518770271928</v>
       </c>
       <c r="D12" s="0">
-        <v>0.024721687652946581</v>
+        <v>0.0034518378058760167</v>
       </c>
       <c r="E12" s="0">
         <v>1.2211103456711071e-07</v>
@@ -2312,7 +2510,7 @@
         <v>0.085441791387548371</v>
       </c>
       <c r="D13" s="0">
-        <v>0.099175662356202884</v>
+        <v>0.0081450867665097543</v>
       </c>
       <c r="E13" s="0">
         <v>7.8952503682134265e-07</v>
@@ -2329,7 +2527,7 @@
         <v>0.050642494068408379</v>
       </c>
       <c r="D14" s="0">
-        <v>0.025426524320007103</v>
+        <v>0.010173355617100789</v>
       </c>
       <c r="E14" s="0">
         <v>4.4677009184411504e-11</v>
@@ -2347,22 +2545,22 @@
     <col min="1" max="1" width="7.85546875" customWidth="true"/>
     <col min="2" max="2" width="12.7109375" customWidth="true"/>
     <col min="3" max="3" width="11.7109375" customWidth="true"/>
-    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>79</v>
+        <v>135</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>80</v>
+        <v>136</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -2379,7 +2577,7 @@
         <v>1.5336895236345123</v>
       </c>
       <c r="D2" s="0">
-        <v>1.4440969626615074</v>
+        <v>1.4675826035160828</v>
       </c>
       <c r="E2" s="0">
         <v>1.1438307958041567</v>
@@ -2396,7 +2594,7 @@
         <v>1.0996958454837389</v>
       </c>
       <c r="D3" s="0">
-        <v>1.3387601597193344</v>
+        <v>0.78707328071411398</v>
       </c>
       <c r="E3" s="0">
         <v>2.0007844145255982</v>
@@ -2413,7 +2611,7 @@
         <v>1.4651793487860167</v>
       </c>
       <c r="D4" s="0">
-        <v>1.7986121491619631</v>
+        <v>0.98022368407427884</v>
       </c>
       <c r="E4" s="0">
         <v>2.5487933810041188</v>
@@ -2430,7 +2628,7 @@
         <v>1.6145440396135229</v>
       </c>
       <c r="D5" s="0">
-        <v>1.9275693004963792</v>
+        <v>0.73127142985848537</v>
       </c>
       <c r="E5" s="0">
         <v>2.6333853691182521</v>
@@ -2447,7 +2645,7 @@
         <v>2.0373444465812938</v>
       </c>
       <c r="D6" s="0">
-        <v>2.0596311866574153</v>
+        <v>0.98019605881960659</v>
       </c>
       <c r="E6" s="0">
         <v>3.0563453096889193</v>
@@ -2464,7 +2662,7 @@
         <v>2.4862695491450117</v>
       </c>
       <c r="D7" s="0">
-        <v>2.5918754868357357</v>
+        <v>1.3455555465822089</v>
       </c>
       <c r="E7" s="0">
         <v>4.1486853301192559</v>
@@ -2481,7 +2679,7 @@
         <v>2.2473902473902472</v>
       </c>
       <c r="D8" s="0">
-        <v>2.8511368511368502</v>
+        <v>1.56027456027456</v>
       </c>
       <c r="E8" s="0">
         <v>4.2112098430731804</v>
@@ -2498,7 +2696,7 @@
         <v>2.5027180587844589</v>
       </c>
       <c r="D9" s="0">
-        <v>2.7151066713241865</v>
+        <v>1.6709349006952003</v>
       </c>
       <c r="E9" s="0">
         <v>4.0567375169517215</v>
@@ -2515,7 +2713,7 @@
         <v>2.0378755618980122</v>
       </c>
       <c r="D10" s="0">
-        <v>2.3244951598062875</v>
+        <v>1.418642900293837</v>
       </c>
       <c r="E10" s="0">
         <v>3.9537559662040795</v>
@@ -2532,7 +2730,7 @@
         <v>1.744535917580917</v>
       </c>
       <c r="D11" s="0">
-        <v>1.8264579275673956</v>
+        <v>1.7525938202025382</v>
       </c>
       <c r="E11" s="0">
         <v>3.1438931878746499</v>
@@ -2549,7 +2747,7 @@
         <v>1.6738206443413512</v>
       </c>
       <c r="D12" s="0">
-        <v>1.4480494876627501</v>
+        <v>1.8968440790319758</v>
       </c>
       <c r="E12" s="0">
         <v>2.8237515995029057</v>
@@ -2566,7 +2764,7 @@
         <v>1.2281292025994892</v>
       </c>
       <c r="D13" s="0">
-        <v>1.1949872230996048</v>
+        <v>1.7765351652673878</v>
       </c>
       <c r="E13" s="0">
         <v>2.6575886279450525</v>
@@ -2583,7 +2781,7 @@
         <v>1.3257457058277033</v>
       </c>
       <c r="D14" s="0">
-        <v>1.44259598022601</v>
+        <v>1.7474645973804379</v>
       </c>
       <c r="E14" s="0">
         <v>3.4340332928975501</v>
@@ -2607,16 +2805,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>83</v>
+        <v>139</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>84</v>
+        <v>140</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>86</v>
+        <v>142</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -2633,7 +2831,7 @@
         <v>0.79575825825825841</v>
       </c>
       <c r="D2" s="0">
-        <v>0.50505721479054821</v>
+        <v>0.49927192040525381</v>
       </c>
       <c r="E2" s="0">
         <v>0.36063063063063067</v>
@@ -2650,7 +2848,7 @@
         <v>0.38835485485485494</v>
       </c>
       <c r="D3" s="0">
-        <v>0.45714664664664667</v>
+        <v>0.10870070070070073</v>
       </c>
       <c r="E3" s="0">
         <v>1.5484009009009014</v>
@@ -2667,7 +2865,7 @@
         <v>0.67179548731121053</v>
       </c>
       <c r="D4" s="0">
-        <v>0.88759362507161221</v>
+        <v>0.11234326150049424</v>
       </c>
       <c r="E4" s="0">
         <v>2.4934459459459464</v>
@@ -2684,7 +2882,7 @@
         <v>1.0831128949462281</v>
       </c>
       <c r="D5" s="0">
-        <v>1.1927328033161371</v>
+        <v>0.10523571006904341</v>
       </c>
       <c r="E5" s="0">
         <v>3.2241271271271255</v>
@@ -2701,7 +2899,7 @@
         <v>1.9614326679620799</v>
       </c>
       <c r="D6" s="0">
-        <v>1.5105909438850613</v>
+        <v>0.15847200141317788</v>
       </c>
       <c r="E6" s="0">
         <v>4.6041391391391393</v>
@@ -2718,7 +2916,7 @@
         <v>2.3403721855188508</v>
       </c>
       <c r="D7" s="0">
-        <v>2.0604970503837174</v>
+        <v>0.34601138471805132</v>
       </c>
       <c r="E7" s="0">
         <v>7.1557107107107125</v>
@@ -2735,7 +2933,7 @@
         <v>1.911840262030738</v>
       </c>
       <c r="D8" s="0">
-        <v>2.2283001709192178</v>
+        <v>0.37911363744697074</v>
       </c>
       <c r="E8" s="0">
         <v>6.985716716716718</v>
@@ -2752,7 +2950,7 @@
         <v>1.844060497997998</v>
       </c>
       <c r="D9" s="0">
-        <v>2.0533987737737744</v>
+        <v>0.48210535535535548</v>
       </c>
       <c r="E9" s="0">
         <v>6.0321136136136158</v>
@@ -2769,7 +2967,7 @@
         <v>1.4191883301741461</v>
       </c>
       <c r="D10" s="0">
-        <v>1.6329147374324682</v>
+        <v>0.52809325637694404</v>
       </c>
       <c r="E10" s="0">
         <v>6.1242572572572591</v>
@@ -2786,7 +2984,7 @@
         <v>0.94586106106106127</v>
       </c>
       <c r="D11" s="0">
-        <v>1.0645101101101095</v>
+        <v>0.75079739739739748</v>
       </c>
       <c r="E11" s="0">
         <v>4.5169491881818908</v>
@@ -2803,7 +3001,7 @@
         <v>0.78555605993590483</v>
       </c>
       <c r="D12" s="0">
-        <v>0.61183796975269855</v>
+        <v>1.0794662026367454</v>
       </c>
       <c r="E12" s="0">
         <v>3.8483844742178079</v>
@@ -2820,7 +3018,7 @@
         <v>0.54708334350610788</v>
       </c>
       <c r="D13" s="0">
-        <v>0.41481329296776448</v>
+        <v>1.2167355322802473</v>
       </c>
       <c r="E13" s="0">
         <v>3.6640834952599661</v>
@@ -2837,7 +3035,7 @@
         <v>0.52295456995456979</v>
       </c>
       <c r="D14" s="0">
-        <v>0.38408701008701007</v>
+        <v>1.1030324940324943</v>
       </c>
       <c r="E14" s="0">
         <v>4.8779485618952272</v>
@@ -2861,16 +3059,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>87</v>
+        <v>143</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>88</v>
+        <v>144</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>90</v>
+        <v>146</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -2885,7 +3083,7 @@
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0">
-        <v>11.410604684127918</v>
+        <v>10.746956888314287</v>
       </c>
       <c r="E2" s="0"/>
     </row>
@@ -2898,7 +3096,7 @@
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0">
-        <v>37.370084988860611</v>
+        <v>31.926983769247272</v>
       </c>
       <c r="E3" s="0"/>
     </row>
@@ -2911,7 +3109,7 @@
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0">
-        <v>60.549607202022173</v>
+        <v>53.423469206462869</v>
       </c>
       <c r="E4" s="0"/>
     </row>
@@ -2924,7 +3122,7 @@
       </c>
       <c r="C5" s="0"/>
       <c r="D5" s="0">
-        <v>75.123852494354139</v>
+        <v>66.850196024913373</v>
       </c>
       <c r="E5" s="0"/>
     </row>
@@ -2937,7 +3135,7 @@
       </c>
       <c r="C6" s="0"/>
       <c r="D6" s="0">
-        <v>82.711286382383662</v>
+        <v>74.532940054928844</v>
       </c>
       <c r="E6" s="0"/>
     </row>
@@ -2950,7 +3148,7 @@
       </c>
       <c r="C7" s="0"/>
       <c r="D7" s="0">
-        <v>85.586291430282813</v>
+        <v>76.801480936934837</v>
       </c>
       <c r="E7" s="0"/>
     </row>
@@ -2963,7 +3161,7 @@
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0">
-        <v>67.160086894315981</v>
+        <v>56.865349564419517</v>
       </c>
       <c r="E8" s="0"/>
     </row>
@@ -2976,7 +3174,7 @@
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0">
-        <v>46.184980846523018</v>
+        <v>35.358338665233973</v>
       </c>
       <c r="E9" s="0"/>
     </row>
@@ -2989,7 +3187,7 @@
       </c>
       <c r="C10" s="0"/>
       <c r="D10" s="0">
-        <v>42.421240880875956</v>
+        <v>30.851117708637446</v>
       </c>
       <c r="E10" s="0"/>
     </row>
@@ -3002,7 +3200,7 @@
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0">
-        <v>42.926118097596671</v>
+        <v>38.90790311515029</v>
       </c>
       <c r="E11" s="0"/>
     </row>
@@ -3015,7 +3213,7 @@
       </c>
       <c r="C12" s="0"/>
       <c r="D12" s="0">
-        <v>50.814808030159334</v>
+        <v>48.214967871429096</v>
       </c>
       <c r="E12" s="0"/>
     </row>
@@ -3028,7 +3226,7 @@
       </c>
       <c r="C13" s="0"/>
       <c r="D13" s="0">
-        <v>73.483807705387193</v>
+        <v>76.179223584738793</v>
       </c>
       <c r="E13" s="0"/>
     </row>
@@ -3041,7 +3239,7 @@
       </c>
       <c r="C14" s="0"/>
       <c r="D14" s="0">
-        <v>63.41597791157303</v>
+        <v>67.707593232564435</v>
       </c>
       <c r="E14" s="0"/>
     </row>
@@ -3063,16 +3261,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>92</v>
+        <v>148</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>93</v>
+        <v>149</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>94</v>
+        <v>150</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -3087,7 +3285,7 @@
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0">
-        <v>6.1031033074175696</v>
+        <v>6.2980661980671186</v>
       </c>
       <c r="E2" s="0"/>
     </row>
@@ -3100,7 +3298,7 @@
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0">
-        <v>25.224455369473958</v>
+        <v>24.8091184013266</v>
       </c>
       <c r="E3" s="0"/>
     </row>
@@ -3113,7 +3311,7 @@
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0">
-        <v>52.430884494124143</v>
+        <v>52.891107281147555</v>
       </c>
       <c r="E4" s="0"/>
     </row>
@@ -3126,7 +3324,7 @@
       </c>
       <c r="C5" s="0"/>
       <c r="D5" s="0">
-        <v>77.546385236796198</v>
+        <v>75.535672407987107</v>
       </c>
       <c r="E5" s="0"/>
     </row>
@@ -3139,7 +3337,7 @@
       </c>
       <c r="C6" s="0"/>
       <c r="D6" s="0">
-        <v>99.183696300707595</v>
+        <v>95.061417187438167</v>
       </c>
       <c r="E6" s="0"/>
     </row>
@@ -3152,7 +3350,7 @@
       </c>
       <c r="C7" s="0"/>
       <c r="D7" s="0">
-        <v>140.58760642256556</v>
+        <v>136.58475749508003</v>
       </c>
       <c r="E7" s="0"/>
     </row>
@@ -3165,7 +3363,7 @@
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0">
-        <v>153.65472171422394</v>
+        <v>145.26354252364533</v>
       </c>
       <c r="E8" s="0"/>
     </row>
@@ -3178,7 +3376,7 @@
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0">
-        <v>119.73137405098797</v>
+        <v>117.46610374748606</v>
       </c>
       <c r="E9" s="0"/>
     </row>
@@ -3191,7 +3389,7 @@
       </c>
       <c r="C10" s="0"/>
       <c r="D10" s="0">
-        <v>90.981566486332298</v>
+        <v>89.984777084976201</v>
       </c>
       <c r="E10" s="0"/>
     </row>
@@ -3204,7 +3402,7 @@
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0">
-        <v>64.65483517296525</v>
+        <v>64.269397588158597</v>
       </c>
       <c r="E11" s="0"/>
     </row>
@@ -3217,7 +3415,7 @@
       </c>
       <c r="C12" s="0"/>
       <c r="D12" s="0">
-        <v>65.80135888438528</v>
+        <v>54.638505398683051</v>
       </c>
       <c r="E12" s="0"/>
     </row>
@@ -3230,7 +3428,7 @@
       </c>
       <c r="C13" s="0"/>
       <c r="D13" s="0">
-        <v>134.65738354268336</v>
+        <v>144.03080300000533</v>
       </c>
       <c r="E13" s="0"/>
     </row>
@@ -3243,7 +3441,7 @@
       </c>
       <c r="C14" s="0"/>
       <c r="D14" s="0">
-        <v>112.63311121604835</v>
+        <v>151.314966414271</v>
       </c>
       <c r="E14" s="0"/>
     </row>
@@ -3265,16 +3463,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>95</v>
+        <v>151</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>96</v>
+        <v>152</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>98</v>
+        <v>154</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -3289,7 +3487,7 @@
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0">
-        <v>0.0097006865624662177</v>
+        <v>0.013175905285370271</v>
       </c>
       <c r="E2" s="0"/>
     </row>
@@ -3302,7 +3500,7 @@
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0">
-        <v>3.8421871719685951e-08</v>
+        <v>5.4222199839313927e-07</v>
       </c>
       <c r="E3" s="0"/>
     </row>
@@ -3315,7 +3513,7 @@
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0">
-        <v>4.485577201150436e-13</v>
+        <v>1.4892225284090346e-11</v>
       </c>
       <c r="E4" s="0"/>
     </row>
@@ -3328,7 +3526,7 @@
       </c>
       <c r="C5" s="0"/>
       <c r="D5" s="0">
-        <v>3.4084858466961797e-16</v>
+        <v>2.0161017616588476e-14</v>
       </c>
       <c r="E5" s="0"/>
     </row>
@@ -3341,7 +3539,7 @@
       </c>
       <c r="C6" s="0"/>
       <c r="D6" s="0">
-        <v>8.0418038451435731e-18</v>
+        <v>4.5625306611798857e-16</v>
       </c>
       <c r="E6" s="0"/>
     </row>
@@ -3354,7 +3552,7 @@
       </c>
       <c r="C7" s="0"/>
       <c r="D7" s="0">
-        <v>1.9422421898629016e-18</v>
+        <v>1.4891670673398467e-16</v>
       </c>
       <c r="E7" s="0"/>
     </row>
@@ -3367,7 +3565,7 @@
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0">
-        <v>1.7305974918729271e-14</v>
+        <v>2.7457148787249849e-12</v>
       </c>
       <c r="E8" s="0"/>
     </row>
@@ -3380,7 +3578,7 @@
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0">
-        <v>5.1804166535037941e-10</v>
+        <v>1.0233396476415416e-07</v>
       </c>
       <c r="E9" s="0"/>
     </row>
@@ -3393,7 +3591,7 @@
       </c>
       <c r="C10" s="0"/>
       <c r="D10" s="0">
-        <v>3.2656853580886856e-09</v>
+        <v>9.136698425394088e-07</v>
       </c>
       <c r="E10" s="0"/>
     </row>
@@ -3406,7 +3604,7 @@
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0">
-        <v>2.5515146534981529e-09</v>
+        <v>1.8154139683718205e-08</v>
       </c>
       <c r="E11" s="0"/>
     </row>
@@ -3419,7 +3617,7 @@
       </c>
       <c r="C12" s="0"/>
       <c r="D12" s="0">
-        <v>5.3573172621621168e-11</v>
+        <v>1.9165774576619879e-10</v>
       </c>
       <c r="E12" s="0"/>
     </row>
@@ -3432,7 +3630,7 @@
       </c>
       <c r="C13" s="0"/>
       <c r="D13" s="0">
-        <v>7.6563837316894364e-16</v>
+        <v>2.0246168078350906e-16</v>
       </c>
       <c r="E13" s="0"/>
     </row>
@@ -3445,7 +3643,7 @@
       </c>
       <c r="C14" s="0"/>
       <c r="D14" s="0">
-        <v>1.0942789073034149e-13</v>
+        <v>1.3213550866918925e-14</v>
       </c>
       <c r="E14" s="0"/>
     </row>
@@ -3467,16 +3665,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>100</v>
+        <v>156</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>101</v>
+        <v>157</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -3491,7 +3689,7 @@
       </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0">
-        <v>0.013494470094551554</v>
+        <v>0.012086975788492424</v>
       </c>
       <c r="E2" s="0"/>
     </row>
@@ -3504,7 +3702,7 @@
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0">
-        <v>5.1030995221069119e-07</v>
+        <v>6.3297330811478278e-07</v>
       </c>
       <c r="E3" s="0"/>
     </row>
@@ -3517,7 +3715,7 @@
       </c>
       <c r="C4" s="0"/>
       <c r="D4" s="0">
-        <v>4.4565984665268264e-13</v>
+        <v>3.5256216948104571e-13</v>
       </c>
       <c r="E4" s="0"/>
     </row>
@@ -3530,7 +3728,7 @@
       </c>
       <c r="C5" s="0"/>
       <c r="D5" s="0">
-        <v>1.2964185871991937e-18</v>
+        <v>3.5886453558667183e-18</v>
       </c>
       <c r="E5" s="0"/>
     </row>
@@ -3543,7 +3741,7 @@
       </c>
       <c r="C6" s="0"/>
       <c r="D6" s="0">
-        <v>2.3013383298971414e-23</v>
+        <v>1.8456919995877228e-22</v>
       </c>
       <c r="E6" s="0"/>
     </row>
@@ -3556,7 +3754,7 @@
       </c>
       <c r="C7" s="0"/>
       <c r="D7" s="0">
-        <v>1.9802483301511833e-32</v>
+        <v>1.4863196789861074e-31</v>
       </c>
       <c r="E7" s="0"/>
     </row>
@@ -3569,7 +3767,7 @@
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0">
-        <v>2.7554108926037584e-35</v>
+        <v>1.8808075619485983e-33</v>
       </c>
       <c r="E8" s="0"/>
     </row>
@@ -3582,7 +3780,7 @@
       </c>
       <c r="C9" s="0"/>
       <c r="D9" s="0">
-        <v>7.2434271564687894e-28</v>
+        <v>2.2694562980612245e-27</v>
       </c>
       <c r="E9" s="0"/>
     </row>
@@ -3595,7 +3793,7 @@
       </c>
       <c r="C10" s="0"/>
       <c r="D10" s="0">
-        <v>1.4501680882865048e-21</v>
+        <v>2.3999954778645826e-21</v>
       </c>
       <c r="E10" s="0"/>
     </row>
@@ -3608,7 +3806,7 @@
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0">
-        <v>8.9237048816151297e-16</v>
+        <v>1.0851826065378379e-15</v>
       </c>
       <c r="E11" s="0"/>
     </row>
@@ -3621,7 +3819,7 @@
       </c>
       <c r="C12" s="0"/>
       <c r="D12" s="0">
-        <v>4.9873835648143897e-16</v>
+        <v>1.4486917793812948e-13</v>
       </c>
       <c r="E12" s="0"/>
     </row>
@@ -3634,7 +3832,7 @@
       </c>
       <c r="C13" s="0"/>
       <c r="D13" s="0">
-        <v>3.9235417411813785e-31</v>
+        <v>3.4982933680931276e-33</v>
       </c>
       <c r="E13" s="0"/>
     </row>
@@ -3647,7 +3845,7 @@
       </c>
       <c r="C14" s="0"/>
       <c r="D14" s="0">
-        <v>2.5963539838610194e-26</v>
+        <v>8.9443225878367405e-35</v>
       </c>
       <c r="E14" s="0"/>
     </row>
@@ -3669,16 +3867,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>103</v>
+        <v>159</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>104</v>
+        <v>160</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>105</v>
+        <v>161</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>4</v>
@@ -3695,7 +3893,7 @@
         <v>9.974381445021212</v>
       </c>
       <c r="D2" s="0">
-        <v>5.8185486540013702</v>
+        <v>6.2564441246887696</v>
       </c>
       <c r="E2" s="0">
         <v>2.2586231601201741</v>
@@ -3712,7 +3910,7 @@
         <v>4.4385055888523066</v>
       </c>
       <c r="D3" s="0">
-        <v>7.7449740536156311</v>
+        <v>4.7876632015097966</v>
       </c>
       <c r="E3" s="0">
         <v>5.6669440562861251</v>
@@ -3729,7 +3927,7 @@
         <v>7.1508145507835081</v>
       </c>
       <c r="D4" s="0">
-        <v>8.7905577328913882</v>
+        <v>5.1121989556372291</v>
       </c>
       <c r="E4" s="0">
         <v>4.9913330483747647</v>
@@ -3746,7 +3944,7 @@
         <v>8.0349533194253873</v>
       </c>
       <c r="D5" s="0">
-        <v>6.8471783334848215</v>
+        <v>4.8635225185416084</v>
       </c>
       <c r="E5" s="0">
         <v>8.9306938635495463</v>
@@ -3763,7 +3961,7 @@
         <v>6.6306018079982678</v>
       </c>
       <c r="D6" s="0">
-        <v>6.3598547741453011</v>
+        <v>4.7525023013450038</v>
       </c>
       <c r="E6" s="0">
         <v>8.6425707604296793</v>
@@ -3780,7 +3978,7 @@
         <v>6.6359314644677152</v>
       </c>
       <c r="D7" s="0">
-        <v>5.411967904524567</v>
+        <v>4.6909661526226873</v>
       </c>
       <c r="E7" s="0">
         <v>13.370425538638409</v>
@@ -3797,7 +3995,7 @@
         <v>7.5513340545422425</v>
       </c>
       <c r="D8" s="0">
-        <v>4.30418038698435</v>
+        <v>3.5981870312828961</v>
       </c>
       <c r="E8" s="0">
         <v>15.308569135295734</v>
@@ -3814,7 +4012,7 @@
         <v>6.4057179467690482</v>
       </c>
       <c r="D9" s="0">
-        <v>3.8952432055775441</v>
+        <v>3.6764198802672658</v>
       </c>
       <c r="E9" s="0">
         <v>15.403077006867361</v>
@@ -3831,7 +4029,7 @@
         <v>4.9139121523609317</v>
       </c>
       <c r="D10" s="0">
-        <v>3.2912492534791205</v>
+        <v>3.3229000086124634</v>
       </c>
       <c r="E10" s="0">
         <v>12.56871204259436</v>
@@ -3848,7 +4046,7 @@
         <v>3.1932905514201151</v>
       </c>
       <c r="D11" s="0">
-        <v>3.9856300418531525</v>
+        <v>3.3412602006674734</v>
       </c>
       <c r="E11" s="0">
         <v>10.265251123660747</v>
@@ -3865,7 +4063,7 @@
         <v>3.6656995525416329</v>
       </c>
       <c r="D12" s="0">
-        <v>5.4656044118402711</v>
+        <v>6.3255202286667505</v>
       </c>
       <c r="E12" s="0">
         <v>10.034027813502727</v>
@@ -3882,7 +4080,7 @@
         <v>3.168181664250092</v>
       </c>
       <c r="D13" s="0">
-        <v>6.351802400068089</v>
+        <v>4.1132954303778044</v>
       </c>
       <c r="E13" s="0">
         <v>12.330090161270089</v>
@@ -3899,7 +4097,7 @@
         <v>3.7161563688265318</v>
       </c>
       <c r="D14" s="0">
-        <v>5.566329221892925</v>
+        <v>4.1963859811454984</v>
       </c>
       <c r="E14" s="0">
         <v>11.314303718961998</v>

</xml_diff>